<commit_message>
Extend Excel path with Buyer ID and Cost Center; 22/22 tests pass
- excel_parser.py: recognise "Buyer ID" / "Cost Center" (and aliases) from
  Excel PO header rows and emit them in the structured text so POExtractor
  picks them up; the full pipeline now works for both text and Excel uploads.
- create_sample_excel.py: add Buyer ID (BUY-001) and Cost Center (CC-MW-100)
  rows to the happy-path Excel; reduce line quantities to stay within pricing
  policy; regenerate both sample-data/US-01/ Excel files.
- test_pipeline.py: add Excel happy-path case; harness now covers 22 cases
  (text + Excel paths, all stories, happy + every exception type).

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/sample-data/US-01/sample-po-happy-path.xlsx
+++ b/sample-data/US-01/sample-po-happy-path.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Purchase Order" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purchase Order" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -510,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -580,233 +580,259 @@
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Contact Person</t>
+          <t>Buyer ID</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>John Miller</t>
+          <t>BUY-001</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Contract Reference</t>
+          <t>Cost Center</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>CONTRACT-ACME-2026-007</t>
+          <t>CC-MW-100</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Payment Terms</t>
+          <t>Contact Person</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Net 30</t>
+          <t>John Miller</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Ship To</t>
+          <t>Contract Reference</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Acme Industrial – Chicago Warehouse, 4500 West Diversey Ave, Chicago IL 60639</t>
+          <t>CONTRACT-ACME-2026-007</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>ZIP</t>
+          <t>Payment Terms</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>60639</t>
+          <t>Net 30</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Delivery Date</t>
+          <t>Ship To</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>15 July 2026</t>
+          <t>Acme Industrial - Chicago Warehouse, 4500 West Diversey Ave, Chicago IL 60639</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
+          <t>ZIP</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>60639</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Delivery Date</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>15 July 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
           <t>Delivery Instructions</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>Deliver to Dock 3. Forklift required. Call 312-555-0199 before arrival.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="26" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="16" ht="26" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Line</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>SKU</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>UOM</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>Unit Price</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="G16" s="4" t="inlineStr">
         <is>
           <t>Line Total</t>
         </is>
-      </c>
-    </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>SKU-STL-4520</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>Carbon Steel Pipe 4 inch SCH40</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="n">
-        <v>500</v>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>FT</t>
-        </is>
-      </c>
-      <c r="F15" s="7" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="G15" s="7" t="n">
-        <v>5400</v>
-      </c>
-    </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>SKU-FLG-3010</t>
-        </is>
-      </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>Stainless Steel Flange 3 inch 150LB</t>
-        </is>
-      </c>
-      <c r="D16" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>EA</t>
-        </is>
-      </c>
-      <c r="F16" s="10" t="n">
-        <v>76</v>
-      </c>
-      <c r="G16" s="10" t="n">
-        <v>6080</v>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>SKU-STL-4520</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>Carbon Steel Pipe 4 inch SCH40</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>200</v>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="G17" s="7" t="n">
+        <v>2160</v>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>SKU-FLG-3010</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Stainless Steel Flange 3 inch 150LB</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="F18" s="10" t="n">
+        <v>39.5</v>
+      </c>
+      <c r="G18" s="10" t="n">
+        <v>3160</v>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>SKU-VLV-2201</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>Ball Valve 2 inch Full Port CS</t>
         </is>
       </c>
-      <c r="D17" s="5" t="n">
+      <c r="D19" s="5" t="n">
         <v>25</v>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>EA</t>
         </is>
       </c>
-      <c r="F17" s="7" t="n">
-        <v>185</v>
-      </c>
-      <c r="G17" s="7" t="n">
-        <v>4625</v>
-      </c>
-    </row>
-    <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="11" t="inlineStr">
+      <c r="F19" s="7" t="n">
+        <v>80</v>
+      </c>
+      <c r="G19" s="7" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="11" t="inlineStr">
         <is>
           <t>ORDER TOTAL</t>
         </is>
       </c>
-      <c r="G18" s="12" t="n">
-        <v>16105</v>
+      <c r="G20" s="12" t="n">
+        <v>7320</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="15">
     <mergeCell ref="B3:G3"/>
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="B10:G10"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="B5:G5"/>
+    <mergeCell ref="B14:G14"/>
     <mergeCell ref="B9:G9"/>
     <mergeCell ref="B8:G8"/>
     <mergeCell ref="B4:G4"/>
     <mergeCell ref="B12:G12"/>
-    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="B13:G13"/>
+    <mergeCell ref="A20:F20"/>
     <mergeCell ref="B7:G7"/>
     <mergeCell ref="B11:G11"/>
     <mergeCell ref="B6:G6"/>

</xml_diff>